<commit_message>
Agrega 3 plantillas Excel, 8 documentos Word, vistas previas, portadas y paquetes ZIP
Corrige etiquetas cortadas, retención IMSS en nómina y mejor opción en el cuadro comparativo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/plantillas/1_Contabilidad_y_Finanzas/04_Cuentas_por_Cobrar.xlsx
+++ b/plantillas/1_Contabilidad_y_Finanzas/04_Cuentas_por_Cobrar.xlsx
@@ -512,12 +512,12 @@
   <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10.05" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18.1" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>

</xml_diff>